<commit_message>
Add ChemOnt classification enricher
Expose classified_by for chemical entities and add a local ChemOnt enricher that looks up the Zenodo ClassyFire/ChemOnt table by InChIKey. The new prepare-chemont command can materialize the large TSV release as an indexed DuckDB database for point lookups or as Parquet for scan-oriented workflows.

Regenerated LinkML artifacts and added tests for DuckDB, Parquet, CLI, and registry coverage.

@dragon-ai-agent
</commit_message>
<xml_diff>
--- a/schema/excel/chemrof.xlsx
+++ b/schema/excel/chemrof.xlsx
@@ -1351,7 +1351,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1497,20 +1497,25 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -1527,7 +1532,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1673,20 +1678,25 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -1703,7 +1713,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AC1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1829,20 +1839,25 @@
       </c>
       <c r="Y1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -1859,7 +1874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2005,20 +2020,25 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -2071,7 +2091,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2217,20 +2237,25 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -2247,7 +2272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2393,20 +2418,25 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -2423,7 +2453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ1"/>
+  <dimension ref="A1:AK1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2589,20 +2619,25 @@
       </c>
       <c r="AG1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -2619,7 +2654,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD1"/>
+  <dimension ref="A1:AE1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2755,20 +2790,25 @@
       </c>
       <c r="AA1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -2785,7 +2825,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ1"/>
+  <dimension ref="A1:AK1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2951,20 +2991,25 @@
       </c>
       <c r="AG1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -2981,7 +3026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ1"/>
+  <dimension ref="A1:AK1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3147,20 +3192,25 @@
       </c>
       <c r="AG1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -3177,7 +3227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3298,20 +3348,25 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -3328,7 +3383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3449,20 +3504,25 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -3479,7 +3539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3600,20 +3660,25 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -3630,7 +3695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3751,20 +3816,25 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -3817,7 +3887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3938,20 +4008,25 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -3968,7 +4043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4109,20 +4184,25 @@
       </c>
       <c r="AB1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -4139,7 +4219,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4285,20 +4365,25 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -4315,7 +4400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG1"/>
+  <dimension ref="A1:AH1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4466,20 +4551,25 @@
       </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -4496,7 +4586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4617,20 +4707,25 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -4647,7 +4742,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AC1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4773,20 +4868,25 @@
       </c>
       <c r="Y1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -4803,7 +4903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AC1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4929,20 +5029,25 @@
       </c>
       <c r="Y1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -4959,7 +5064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AC1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5085,20 +5190,25 @@
       </c>
       <c r="Y1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -5115,7 +5225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AC1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5241,20 +5351,25 @@
       </c>
       <c r="Y1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -5271,7 +5386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5392,20 +5507,25 @@
       </c>
       <c r="X1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -5468,7 +5588,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5614,20 +5734,25 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -5644,7 +5769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5790,20 +5915,25 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -5820,7 +5950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ1"/>
+  <dimension ref="A1:AK1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5981,25 +6111,30 @@
       </c>
       <c r="AF1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>elemental_charge</t>
         </is>
@@ -6021,7 +6156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ1"/>
+  <dimension ref="A1:AK1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6182,25 +6317,30 @@
       </c>
       <c r="AF1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>elemental_charge</t>
         </is>
@@ -6222,7 +6362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ1"/>
+  <dimension ref="A1:AK1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6383,25 +6523,30 @@
       </c>
       <c r="AF1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>elemental_charge</t>
         </is>
@@ -6423,7 +6568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH1"/>
+  <dimension ref="A1:AI1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6574,25 +6719,30 @@
       </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>elemental_charge</t>
         </is>
@@ -6614,7 +6764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH1"/>
+  <dimension ref="A1:AI1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6765,25 +6915,30 @@
       </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>elemental_charge</t>
         </is>
@@ -6805,7 +6960,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AH1"/>
+  <dimension ref="A1:AI1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6956,25 +7111,30 @@
       </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>elemental_charge</t>
         </is>
@@ -6996,7 +7156,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7147,15 +7307,20 @@
       </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -7177,7 +7342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7323,15 +7488,20 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -7394,7 +7564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7540,15 +7710,20 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -7565,7 +7740,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7711,15 +7886,20 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -7736,7 +7916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM1"/>
+  <dimension ref="A1:AN1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7922,15 +8102,20 @@
       </c>
       <c r="AK1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -7947,7 +8132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM1"/>
+  <dimension ref="A1:AN1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8133,15 +8318,20 @@
       </c>
       <c r="AK1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -8158,7 +8348,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8309,15 +8499,20 @@
       </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -8334,7 +8529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8485,15 +8680,20 @@
       </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -8510,7 +8710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8661,15 +8861,20 @@
       </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -8686,7 +8891,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8837,15 +9042,20 @@
       </c>
       <c r="AD1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -9508,7 +9718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB1"/>
+  <dimension ref="A1:AC1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9634,20 +9844,25 @@
       </c>
       <c r="Y1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -9664,7 +9879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9810,20 +10025,25 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -9840,7 +10060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9986,20 +10206,25 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -10016,7 +10241,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10162,20 +10387,25 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -10192,7 +10422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10333,20 +10563,25 @@
       </c>
       <c r="AB1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>type</t>
         </is>
@@ -10363,7 +10598,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF1"/>
+  <dimension ref="A1:AG1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10509,20 +10744,25 @@
       </c>
       <c r="AC1" t="inlineStr">
         <is>
+          <t>classified_by</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
           <t>owl_subclass_of</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>type</t>
         </is>

</xml_diff>